<commit_message>
add website price and fixed excel sheet for upload product
</commit_message>
<xml_diff>
--- a/public/sample_file/sample_products.xlsx
+++ b/public/sample_file/sample_products.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="75">
   <si>
     <t>Product Name</t>
   </si>
@@ -50,6 +50,9 @@
     <t>Product Price</t>
   </si>
   <si>
+    <t>Website Price</t>
+  </si>
+  <si>
     <t>Variant Option</t>
   </si>
   <si>
@@ -65,6 +68,18 @@
     <t>Image</t>
   </si>
   <si>
+    <t>3D Model File</t>
+  </si>
+  <si>
+    <t>Product Tags</t>
+  </si>
+  <si>
+    <t>Meta Title</t>
+  </si>
+  <si>
+    <t>Meta Description</t>
+  </si>
+  <si>
     <t>Napa Extra</t>
   </si>
   <si>
@@ -95,6 +110,9 @@
     <t>25</t>
   </si>
   <si>
+    <t>24</t>
+  </si>
+  <si>
     <t>Dose</t>
   </si>
   <si>
@@ -107,79 +125,121 @@
     <t>Paracetamol + Caffeine fast pain relief</t>
   </si>
   <si>
-    <t>napa_extra.jpg</t>
-  </si>
-  <si>
-    <t>Ace Plus</t>
+    <t>napa.jpg</t>
+  </si>
+  <si>
+    <t>napa_model.glb</t>
+  </si>
+  <si>
+    <t>paracetamol, fever, pain relief</t>
+  </si>
+  <si>
+    <t>Napa Extra 500mg/65mg Fast Pain Relief</t>
+  </si>
+  <si>
+    <t>Buy Napa Extra fast pain relief tablets online at the best price.</t>
+  </si>
+  <si>
+    <t>Seclo 20</t>
   </si>
   <si>
     <t>MED-1002</t>
   </si>
   <si>
-    <t>Syrup</t>
+    <t>Capsule</t>
   </si>
   <si>
     <t>Square</t>
   </si>
   <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>21.6</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>Paracetamol 500mg and Caffeine 65mg</t>
-  </si>
-  <si>
-    <t>ace_plus.jpg</t>
-  </si>
-  <si>
-    <t>Premium Cotton Polo Shirt</t>
-  </si>
-  <si>
-    <t>APP-2001</t>
-  </si>
-  <si>
-    <t>Fashion &amp; Apparel</t>
-  </si>
-  <si>
-    <t>Clothing</t>
-  </si>
-  <si>
-    <t>Men Fashion</t>
-  </si>
-  <si>
-    <t>Apex</t>
-  </si>
-  <si>
-    <t>450</t>
+    <t>6</t>
+  </si>
+  <si>
+    <t>16.67</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>6.8</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>Omeprazole 20mg gastric acid reducer</t>
+  </si>
+  <si>
+    <t>seclo.jpg</t>
+  </si>
+  <si>
+    <t>gastric, omeprazole, heartburn</t>
+  </si>
+  <si>
+    <t>Seclo 20 Capsule Square Pharmaceuticals</t>
+  </si>
+  <si>
+    <t>Order Seclo 20mg capsules online for gastric relief.</t>
+  </si>
+  <si>
+    <t>Digital Blood Pressure Monitor</t>
+  </si>
+  <si>
+    <t>DEV-2001</t>
+  </si>
+  <si>
+    <t>Medical Devices</t>
+  </si>
+  <si>
+    <t>Healthcare Devices</t>
+  </si>
+  <si>
+    <t>Monitors</t>
+  </si>
+  <si>
+    <t>Omron</t>
+  </si>
+  <si>
+    <t>2500</t>
   </si>
   <si>
     <t>flat</t>
   </si>
   <si>
-    <t>200</t>
-  </si>
-  <si>
-    <t>650</t>
-  </si>
-  <si>
-    <t>Size | Color</t>
-  </si>
-  <si>
-    <t>S, M, L | Red, Blue, Black</t>
+    <t>500</t>
+  </si>
+  <si>
+    <t>3000</t>
+  </si>
+  <si>
+    <t>2850</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>Standard Cuff, Large Cuff</t>
   </si>
   <si>
     <t>5</t>
   </si>
   <si>
-    <t>100% combed cotton breathable polo shirt with multi size and color</t>
-  </si>
-  <si>
-    <t>polo_shirt.jpg</t>
+    <t>Accurate digital upper arm blood pressure monitor</t>
+  </si>
+  <si>
+    <t>bp_monitor.jpg</t>
+  </si>
+  <si>
+    <t>bp_monitor.glb</t>
+  </si>
+  <si>
+    <t>omron, bp monitor, medical device</t>
+  </si>
+  <si>
+    <t>Omron Digital BP Monitor</t>
+  </si>
+  <si>
+    <t>Buy Omron Upper Arm Digital Blood Pressure Monitor with Warranty.</t>
   </si>
 </sst>
 </file>
@@ -187,7 +247,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -204,6 +264,15 @@
       <u val="none"/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -227,7 +296,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -235,17 +304,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFE2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFE2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFE2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFE2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="3" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="2" numFmtId="0" fillId="0" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -546,13 +648,13 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:P4"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="30.564" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="32.992" bestFit="true" customWidth="true" style="0"/>
     <col min="2" max="2" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="3" max="3" width="20.995" bestFit="true" customWidth="true" style="0"/>
+    <col min="4" max="4" width="20.138" bestFit="true" customWidth="true" style="0"/>
     <col min="5" max="5" width="17.567" bestFit="true" customWidth="true" style="0"/>
     <col min="6" max="6" width="9.283" bestFit="true" customWidth="true" style="0"/>
     <col min="7" max="7" width="17.567" bestFit="true" customWidth="true" style="0"/>
@@ -560,14 +662,19 @@
     <col min="9" max="9" width="24.565" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="18.71" bestFit="true" customWidth="true" style="0"/>
     <col min="11" max="11" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="19.852" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="19.852" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="78.981" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="17.567" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="19.852" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="27.708" bestFit="true" customWidth="true" style="0"/>
+    <col min="15" max="15" width="19.852" bestFit="true" customWidth="true" style="0"/>
+    <col min="16" max="16" width="53.416" bestFit="true" customWidth="true" style="0"/>
+    <col min="17" max="17" width="15.853" bestFit="true" customWidth="true" style="0"/>
+    <col min="18" max="18" width="18.71" bestFit="true" customWidth="true" style="0"/>
+    <col min="19" max="19" width="36.277" bestFit="true" customWidth="true" style="0"/>
+    <col min="20" max="20" width="42.704" bestFit="true" customWidth="true" style="0"/>
+    <col min="21" max="21" width="70.554" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" customHeight="1" ht="28">
+    <row r="1" spans="1:21" customHeight="1" ht="28">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -616,151 +723,209 @@
       <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:16">
-      <c r="A2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" t="s">
+    <row r="2" spans="1:21" customHeight="1" ht="22">
+      <c r="A2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G2" t="s">
+      <c r="B2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="H2" t="s">
+      <c r="C2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I2" t="s">
+      <c r="D2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="J2" t="s">
+      <c r="E2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="K2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L2" t="s">
+      <c r="F2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="M2" t="s">
+      <c r="G2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="N2" t="s">
+      <c r="H2" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="O2" t="s">
+      <c r="I2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="P2" t="s">
+      <c r="J2" s="3" t="s">
         <v>30</v>
       </c>
+      <c r="K2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="O2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="R2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="S2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="3" spans="1:16">
-      <c r="A3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" t="s">
+    <row r="3" spans="1:21" customHeight="1" ht="22">
+      <c r="A3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="J3" t="s">
-        <v>23</v>
-      </c>
-      <c r="K3" t="s">
-        <v>36</v>
-      </c>
-      <c r="L3"/>
-      <c r="M3"/>
-      <c r="N3" t="s">
-        <v>37</v>
-      </c>
-      <c r="O3" t="s">
-        <v>38</v>
-      </c>
-      <c r="P3" t="s">
-        <v>39</v>
+      <c r="E3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
-      <c r="A4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" t="s">
-        <v>43</v>
-      </c>
-      <c r="E4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" t="s">
-        <v>46</v>
-      </c>
-      <c r="I4" t="s">
-        <v>47</v>
-      </c>
-      <c r="J4" t="s">
-        <v>48</v>
-      </c>
-      <c r="K4" t="s">
-        <v>49</v>
-      </c>
-      <c r="L4" t="s">
-        <v>50</v>
-      </c>
-      <c r="M4" t="s">
-        <v>51</v>
-      </c>
-      <c r="N4" t="s">
-        <v>52</v>
-      </c>
-      <c r="O4" t="s">
-        <v>53</v>
-      </c>
-      <c r="P4" t="s">
-        <v>54</v>
+    <row r="4" spans="1:21" customHeight="1" ht="22">
+      <c r="A4" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>